<commit_message>
Day 12 - Populated financial_ratios table
</commit_message>
<xml_diff>
--- a/data/processed/analysis_clean.xlsx
+++ b/data/processed/analysis_clean.xlsx
@@ -1,38 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Narendra\Desktop\nifty100_project\data\processed\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30487410-E1B5-4B81-A7A4-34A01922AD1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="3000" yWindow="3000" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="114">
-  <si>
-    <t>bluestock fintech — nifty 100  |  analysis  |  20 records</t>
-  </si>
-  <si>
-    <t>unnamed: 1</t>
-  </si>
-  <si>
-    <t>unnamed: 2</t>
-  </si>
-  <si>
-    <t>unnamed: 3</t>
-  </si>
-  <si>
-    <t>unnamed: 4</t>
-  </si>
-  <si>
-    <t>unnamed: 5</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="108">
   <si>
     <t>id</t>
   </si>
@@ -361,17 +349,9 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -387,7 +367,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -395,43 +375,33 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -469,7 +439,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -503,6 +473,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -537,9 +508,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -712,448 +684,428 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F22"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:F21"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:6">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" t="s">
+        <v>48</v>
+      </c>
+      <c r="E1" t="s">
+        <v>67</v>
+      </c>
+      <c r="F1" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="B2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D2" t="s">
+        <v>49</v>
+      </c>
+      <c r="E2" t="s">
+        <v>68</v>
+      </c>
+      <c r="F2" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="B3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D3" t="s">
+        <v>50</v>
+      </c>
+      <c r="E3" t="s">
+        <v>69</v>
+      </c>
+      <c r="F3" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="B4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C4" t="s">
+        <v>30</v>
+      </c>
+      <c r="D4" t="s">
+        <v>51</v>
+      </c>
+      <c r="E4" t="s">
+        <v>70</v>
+      </c>
+      <c r="F4" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="B5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C5" t="s">
+        <v>31</v>
+      </c>
+      <c r="D5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E5" t="s">
+        <v>71</v>
+      </c>
+      <c r="F5" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:6">
-      <c r="A2" t="s">
+      <c r="B6" t="s">
+        <v>24</v>
+      </c>
+      <c r="C6" t="s">
+        <v>32</v>
+      </c>
+      <c r="D6" t="s">
+        <v>53</v>
+      </c>
+      <c r="E6" t="s">
+        <v>72</v>
+      </c>
+      <c r="F6" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
         <v>6</v>
       </c>
-      <c r="B2" t="s">
-        <v>27</v>
-      </c>
-      <c r="C2" t="s">
+      <c r="B7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C7" t="s">
         <v>33</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D7" t="s">
         <v>54</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E7" t="s">
         <v>73</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F7" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
-      <c r="A3" t="s">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
         <v>7</v>
       </c>
-      <c r="B3" t="s">
-        <v>28</v>
-      </c>
-      <c r="C3" t="s">
+      <c r="B8" t="s">
+        <v>24</v>
+      </c>
+      <c r="C8" t="s">
         <v>34</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D8" t="s">
         <v>55</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E8" t="s">
         <v>74</v>
       </c>
-      <c r="F3" t="s">
+      <c r="F8" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
-      <c r="A4" t="s">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
         <v>8</v>
       </c>
-      <c r="B4" t="s">
-        <v>29</v>
-      </c>
-      <c r="C4" t="s">
+      <c r="B9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C9" t="s">
         <v>35</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D9" t="s">
         <v>56</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E9" t="s">
         <v>75</v>
       </c>
-      <c r="F4" t="s">
+      <c r="F9" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="5" spans="1:6">
-      <c r="A5" t="s">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
         <v>9</v>
       </c>
-      <c r="B5" t="s">
-        <v>29</v>
-      </c>
-      <c r="C5" t="s">
+      <c r="B10" t="s">
+        <v>25</v>
+      </c>
+      <c r="C10" t="s">
         <v>36</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D10" t="s">
         <v>57</v>
       </c>
-      <c r="E5" t="s">
+      <c r="E10" t="s">
         <v>76</v>
       </c>
-      <c r="F5" t="s">
+      <c r="F10" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
-      <c r="A6" t="s">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
         <v>10</v>
       </c>
-      <c r="B6" t="s">
-        <v>29</v>
-      </c>
-      <c r="C6" t="s">
+      <c r="B11" t="s">
+        <v>25</v>
+      </c>
+      <c r="C11" t="s">
         <v>37</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D11" t="s">
         <v>58</v>
       </c>
-      <c r="E6" t="s">
+      <c r="E11" t="s">
         <v>77</v>
       </c>
-      <c r="F6" t="s">
+      <c r="F11" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="7" spans="1:6">
-      <c r="A7" t="s">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
         <v>11</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B12" t="s">
+        <v>25</v>
+      </c>
+      <c r="C12" t="s">
+        <v>38</v>
+      </c>
+      <c r="D12" t="s">
+        <v>59</v>
+      </c>
+      <c r="E12" t="s">
+        <v>78</v>
+      </c>
+      <c r="F12" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>22</v>
+      </c>
+      <c r="C13" t="s">
+        <v>39</v>
+      </c>
+      <c r="D13" t="s">
+        <v>60</v>
+      </c>
+      <c r="E13" t="s">
+        <v>79</v>
+      </c>
+      <c r="F13" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
+        <v>25</v>
+      </c>
+      <c r="C14" t="s">
+        <v>40</v>
+      </c>
+      <c r="D14" t="s">
+        <v>61</v>
+      </c>
+      <c r="E14" t="s">
+        <v>80</v>
+      </c>
+      <c r="F14" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>22</v>
+      </c>
+      <c r="C15" t="s">
+        <v>41</v>
+      </c>
+      <c r="D15" t="s">
+        <v>62</v>
+      </c>
+      <c r="E15" t="s">
+        <v>81</v>
+      </c>
+      <c r="F15" t="s">
         <v>30</v>
       </c>
-      <c r="C7" t="s">
-        <v>38</v>
-      </c>
-      <c r="D7" t="s">
-        <v>59</v>
-      </c>
-      <c r="E7" t="s">
-        <v>78</v>
-      </c>
-      <c r="F7" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6">
-      <c r="A8" t="s">
-        <v>12</v>
-      </c>
-      <c r="B8" t="s">
-        <v>30</v>
-      </c>
-      <c r="C8" t="s">
-        <v>39</v>
-      </c>
-      <c r="D8" t="s">
-        <v>60</v>
-      </c>
-      <c r="E8" t="s">
-        <v>79</v>
-      </c>
-      <c r="F8" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6">
-      <c r="A9" t="s">
-        <v>13</v>
-      </c>
-      <c r="B9" t="s">
-        <v>30</v>
-      </c>
-      <c r="C9" t="s">
-        <v>40</v>
-      </c>
-      <c r="D9" t="s">
-        <v>61</v>
-      </c>
-      <c r="E9" t="s">
-        <v>80</v>
-      </c>
-      <c r="F9" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6">
-      <c r="A10" t="s">
-        <v>14</v>
-      </c>
-      <c r="B10" t="s">
-        <v>30</v>
-      </c>
-      <c r="C10" t="s">
-        <v>41</v>
-      </c>
-      <c r="D10" t="s">
-        <v>62</v>
-      </c>
-      <c r="E10" t="s">
-        <v>81</v>
-      </c>
-      <c r="F10" t="s">
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>15</v>
+      </c>
+      <c r="B16" t="s">
+        <v>22</v>
+      </c>
+      <c r="C16" t="s">
+        <v>42</v>
+      </c>
+      <c r="D16" t="s">
+        <v>63</v>
+      </c>
+      <c r="E16" t="s">
+        <v>82</v>
+      </c>
+      <c r="F16" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="11" spans="1:6">
-      <c r="A11" t="s">
-        <v>15</v>
-      </c>
-      <c r="B11" t="s">
-        <v>31</v>
-      </c>
-      <c r="C11" t="s">
-        <v>42</v>
-      </c>
-      <c r="D11" t="s">
-        <v>63</v>
-      </c>
-      <c r="E11" t="s">
-        <v>82</v>
-      </c>
-      <c r="F11" t="s">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>16</v>
+      </c>
+      <c r="B17" t="s">
+        <v>26</v>
+      </c>
+      <c r="C17" t="s">
+        <v>43</v>
+      </c>
+      <c r="D17" t="s">
+        <v>64</v>
+      </c>
+      <c r="E17" t="s">
+        <v>83</v>
+      </c>
+      <c r="F17" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="12" spans="1:6">
-      <c r="A12" t="s">
-        <v>16</v>
-      </c>
-      <c r="B12" t="s">
-        <v>31</v>
-      </c>
-      <c r="C12" t="s">
-        <v>43</v>
-      </c>
-      <c r="D12" t="s">
-        <v>64</v>
-      </c>
-      <c r="E12" t="s">
-        <v>83</v>
-      </c>
-      <c r="F12" t="s">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>17</v>
+      </c>
+      <c r="B18" t="s">
+        <v>26</v>
+      </c>
+      <c r="C18" t="s">
+        <v>44</v>
+      </c>
+      <c r="D18" t="s">
+        <v>65</v>
+      </c>
+      <c r="E18" t="s">
+        <v>84</v>
+      </c>
+      <c r="F18" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="13" spans="1:6">
-      <c r="A13" t="s">
-        <v>17</v>
-      </c>
-      <c r="B13" t="s">
-        <v>31</v>
-      </c>
-      <c r="C13" t="s">
-        <v>44</v>
-      </c>
-      <c r="D13" t="s">
-        <v>65</v>
-      </c>
-      <c r="E13" t="s">
-        <v>84</v>
-      </c>
-      <c r="F13" t="s">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>18</v>
+      </c>
+      <c r="B19" t="s">
+        <v>26</v>
+      </c>
+      <c r="C19" t="s">
+        <v>45</v>
+      </c>
+      <c r="D19" t="s">
+        <v>66</v>
+      </c>
+      <c r="E19" t="s">
+        <v>85</v>
+      </c>
+      <c r="F19" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="14" spans="1:6">
-      <c r="A14" t="s">
-        <v>18</v>
-      </c>
-      <c r="B14" t="s">
-        <v>28</v>
-      </c>
-      <c r="C14" t="s">
-        <v>45</v>
-      </c>
-      <c r="D14" t="s">
-        <v>66</v>
-      </c>
-      <c r="E14" t="s">
-        <v>85</v>
-      </c>
-      <c r="F14" t="s">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>19</v>
+      </c>
+      <c r="B20" t="s">
+        <v>26</v>
+      </c>
+      <c r="C20" t="s">
+        <v>46</v>
+      </c>
+      <c r="D20" t="s">
+        <v>56</v>
+      </c>
+      <c r="E20" t="s">
+        <v>86</v>
+      </c>
+      <c r="F20" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="15" spans="1:6">
-      <c r="A15" t="s">
-        <v>19</v>
-      </c>
-      <c r="B15" t="s">
-        <v>31</v>
-      </c>
-      <c r="C15" t="s">
-        <v>46</v>
-      </c>
-      <c r="D15" t="s">
-        <v>67</v>
-      </c>
-      <c r="E15" t="s">
-        <v>86</v>
-      </c>
-      <c r="F15" t="s">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>20</v>
+      </c>
+      <c r="B21" t="s">
+        <v>23</v>
+      </c>
+      <c r="C21" t="s">
+        <v>47</v>
+      </c>
+      <c r="D21" t="s">
+        <v>53</v>
+      </c>
+      <c r="E21" t="s">
+        <v>87</v>
+      </c>
+      <c r="F21" t="s">
         <v>107</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6">
-      <c r="A16" t="s">
-        <v>20</v>
-      </c>
-      <c r="B16" t="s">
-        <v>28</v>
-      </c>
-      <c r="C16" t="s">
-        <v>47</v>
-      </c>
-      <c r="D16" t="s">
-        <v>68</v>
-      </c>
-      <c r="E16" t="s">
-        <v>87</v>
-      </c>
-      <c r="F16" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6">
-      <c r="A17" t="s">
-        <v>21</v>
-      </c>
-      <c r="B17" t="s">
-        <v>28</v>
-      </c>
-      <c r="C17" t="s">
-        <v>48</v>
-      </c>
-      <c r="D17" t="s">
-        <v>69</v>
-      </c>
-      <c r="E17" t="s">
-        <v>88</v>
-      </c>
-      <c r="F17" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6">
-      <c r="A18" t="s">
-        <v>22</v>
-      </c>
-      <c r="B18" t="s">
-        <v>32</v>
-      </c>
-      <c r="C18" t="s">
-        <v>49</v>
-      </c>
-      <c r="D18" t="s">
-        <v>70</v>
-      </c>
-      <c r="E18" t="s">
-        <v>89</v>
-      </c>
-      <c r="F18" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6">
-      <c r="A19" t="s">
-        <v>23</v>
-      </c>
-      <c r="B19" t="s">
-        <v>32</v>
-      </c>
-      <c r="C19" t="s">
-        <v>50</v>
-      </c>
-      <c r="D19" t="s">
-        <v>71</v>
-      </c>
-      <c r="E19" t="s">
-        <v>90</v>
-      </c>
-      <c r="F19" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6">
-      <c r="A20" t="s">
-        <v>24</v>
-      </c>
-      <c r="B20" t="s">
-        <v>32</v>
-      </c>
-      <c r="C20" t="s">
-        <v>51</v>
-      </c>
-      <c r="D20" t="s">
-        <v>72</v>
-      </c>
-      <c r="E20" t="s">
-        <v>91</v>
-      </c>
-      <c r="F20" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6">
-      <c r="A21" t="s">
-        <v>25</v>
-      </c>
-      <c r="B21" t="s">
-        <v>32</v>
-      </c>
-      <c r="C21" t="s">
-        <v>52</v>
-      </c>
-      <c r="D21" t="s">
-        <v>62</v>
-      </c>
-      <c r="E21" t="s">
-        <v>92</v>
-      </c>
-      <c r="F21" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6">
-      <c r="A22" t="s">
-        <v>26</v>
-      </c>
-      <c r="B22" t="s">
-        <v>29</v>
-      </c>
-      <c r="C22" t="s">
-        <v>53</v>
-      </c>
-      <c r="D22" t="s">
-        <v>59</v>
-      </c>
-      <c r="E22" t="s">
-        <v>93</v>
-      </c>
-      <c r="F22" t="s">
-        <v>113</v>
       </c>
     </row>
   </sheetData>

</xml_diff>